<commit_message>
Add SurgExplore to AI roster + viability bins (RISK); 150 companies
</commit_message>
<xml_diff>
--- a/viability-bins.xlsx
+++ b/viability-bins.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -12,7 +12,7 @@
     <sheet name="Companies" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$150</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$151</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,9 +24,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="338">
-  <si>
-    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 149 companies land' chart</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="340">
+  <si>
+    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 150 companies land' chart</t>
   </si>
   <si>
     <t xml:space="preserve">Method: bins are the author's hypotheses about the most probable 2031 outcome, assigned from the master roster (status, funding, notes) combined with public-source research, updated July 28, 2026 after a company-by-company verification pass. Large diversified companies (Intuitive, Medtronic, Stryker, J&amp;J, Olympus, Zeiss, Philips, Brainlab, Accuray, ATEC) are represented as incumbent-platform entries. Bins assess category economics, not team or technology quality; corrections are welcome.</t>
@@ -41,7 +41,7 @@
     <t xml:space="preserve">Companies</t>
   </si>
   <si>
-    <t xml:space="preserve">Share of 149</t>
+    <t xml:space="preserve">Share of 150</t>
   </si>
   <si>
     <t xml:space="preserve">INC</t>
@@ -1038,16 +1038,21 @@
   </si>
   <si>
     <t xml:space="preserve">Operates as a product line of Genesis MedTech rather than an independent company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SurgExplore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grant-stage Bern spin-off (Venture Kick, InnoBooster); cataract video plus EHR analytics with no clearance or disclosed payment path yet; outcome depends on the next financing round</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -1156,24 +1161,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1181,11 +1190,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1302,34 +1311,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1475,176 +1484,176 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A5)</f>
         <v>10</v>
       </c>
-      <c r="D5" s="7" t="n">
-        <f aca="false">C5/149</f>
-        <v>0.0671140939597315</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="D5" s="8" t="n">
+        <f aca="false">C5/150</f>
+        <v>0.0666666666666667</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A6)</f>
         <v>5</v>
       </c>
-      <c r="D6" s="7" t="n">
-        <f aca="false">C6/149</f>
-        <v>0.0335570469798658</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="D6" s="8" t="n">
+        <f aca="false">C6/150</f>
+        <v>0.0333333333333333</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A7)</f>
         <v>9</v>
       </c>
-      <c r="D7" s="7" t="n">
-        <f aca="false">C7/149</f>
-        <v>0.0604026845637584</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="D7" s="8" t="n">
+        <f aca="false">C7/150</f>
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A8)</f>
         <v>33</v>
       </c>
-      <c r="D8" s="7" t="n">
-        <f aca="false">C8/149</f>
-        <v>0.221476510067114</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="D8" s="8" t="n">
+        <f aca="false">C8/150</f>
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A9)</f>
         <v>25</v>
       </c>
-      <c r="D9" s="7" t="n">
-        <f aca="false">C9/149</f>
-        <v>0.167785234899329</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="D9" s="8" t="n">
+        <f aca="false">C9/150</f>
+        <v>0.166666666666667</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A10)</f>
         <v>22</v>
       </c>
-      <c r="D10" s="7" t="n">
-        <f aca="false">C10/149</f>
-        <v>0.147651006711409</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="D10" s="8" t="n">
+        <f aca="false">C10/150</f>
+        <v>0.146666666666667</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A11)</f>
-        <v>35</v>
-      </c>
-      <c r="D11" s="7" t="n">
-        <f aca="false">C11/149</f>
-        <v>0.23489932885906</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <f aca="false">C11/150</f>
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A12)</f>
         <v>10</v>
       </c>
-      <c r="D12" s="7" t="n">
-        <f aca="false">C12/149</f>
-        <v>0.0671140939597315</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="D12" s="8" t="n">
+        <f aca="false">C12/150</f>
+        <v>0.0666666666666667</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="6" t="n">
+      <c r="B13" s="9"/>
+      <c r="C13" s="7" t="n">
         <f aca="false">SUM(C5:C12)</f>
-        <v>149</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <f aca="false">C13/149</f>
+        <v>150</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <f aca="false">C13/150</f>
         <v>1</v>
       </c>
     </row>
@@ -1664,2117 +1673,2131 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D150"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D151"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="110"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="6" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="6" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="6" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="6" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="6" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="6" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
+    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="6" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
+    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="6" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="6" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="6" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="6" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="6" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+    <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D31" s="6" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
+    <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="6" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="6" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="6" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="6" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="6" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D38" s="6" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="D39" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="6" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D41" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="D42" s="6" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D43" s="5" t="s">
+      <c r="D43" s="6" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="s">
+    <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="D44" s="6" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="6" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="D45" s="6" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="6" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="D46" s="6" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="6" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D47" s="5" t="s">
+      <c r="D47" s="6" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="6" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D48" s="5" t="s">
+      <c r="D48" s="6" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="6" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D49" s="5" t="s">
+      <c r="D49" s="6" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="6" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D50" s="5" t="s">
+      <c r="D50" s="6" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="6" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D51" s="5" t="s">
+      <c r="D51" s="6" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="6" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D52" s="5" t="s">
+      <c r="D52" s="6" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B53" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C53" s="6" t="s">
+      <c r="C53" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D53" s="5" t="s">
+      <c r="D53" s="6" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="6" t="s">
+    <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C54" s="6" t="s">
+      <c r="C54" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D54" s="5" t="s">
+      <c r="D54" s="6" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="6" t="s">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="B55" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C55" s="6" t="s">
+      <c r="C55" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D55" s="5" t="s">
+      <c r="D55" s="6" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="6" t="s">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="B56" s="6" t="s">
+      <c r="B56" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C56" s="6" t="s">
+      <c r="C56" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D56" s="5" t="s">
+      <c r="D56" s="6" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="6" t="s">
+    <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="B57" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C57" s="6" t="s">
+      <c r="C57" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D57" s="5" t="s">
+      <c r="D57" s="6" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="6" t="s">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="B58" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C58" s="6" t="s">
+      <c r="C58" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D58" s="5" t="s">
+      <c r="D58" s="6" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="6" t="s">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D59" s="5" t="s">
+      <c r="D59" s="6" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="6" t="s">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="B60" s="6" t="s">
+      <c r="B60" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="C60" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="D60" s="6" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="6" t="s">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="B61" s="6" t="s">
+      <c r="B61" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D61" s="5" t="s">
+      <c r="D61" s="6" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="6" t="s">
+    <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B62" s="6" t="s">
+      <c r="B62" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C62" s="6" t="s">
+      <c r="C62" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="D62" s="6" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="6" t="s">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B63" s="6" t="s">
+      <c r="B63" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C63" s="6" t="s">
+      <c r="C63" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D63" s="5" t="s">
+      <c r="D63" s="6" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="6" t="s">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="B64" s="6" t="s">
+      <c r="B64" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C64" s="6" t="s">
+      <c r="C64" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D64" s="5" t="s">
+      <c r="D64" s="6" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="6" t="s">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="B65" s="6" t="s">
+      <c r="B65" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C65" s="6" t="s">
+      <c r="C65" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D65" s="5" t="s">
+      <c r="D65" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="6" t="s">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="B66" s="6" t="s">
+      <c r="B66" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="C66" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D66" s="5" t="s">
+      <c r="D66" s="6" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="6" t="s">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="B67" s="6" t="s">
+      <c r="B67" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C67" s="6" t="s">
+      <c r="C67" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D67" s="5" t="s">
+      <c r="D67" s="6" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="6" t="s">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="B68" s="6" t="s">
+      <c r="B68" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C68" s="6" t="s">
+      <c r="C68" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D68" s="5" t="s">
+      <c r="D68" s="6" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="6" t="s">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="B69" s="6" t="s">
+      <c r="B69" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C69" s="6" t="s">
+      <c r="C69" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D69" s="5" t="s">
+      <c r="D69" s="6" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="6" t="s">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="B70" s="6" t="s">
+      <c r="B70" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C70" s="6" t="s">
+      <c r="C70" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D70" s="5" t="s">
+      <c r="D70" s="6" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="6" t="s">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="B71" s="6" t="s">
+      <c r="B71" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C71" s="6" t="s">
+      <c r="C71" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D71" s="5" t="s">
+      <c r="D71" s="6" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="6" t="s">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="B72" s="6" t="s">
+      <c r="B72" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C72" s="6" t="s">
+      <c r="C72" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D72" s="5" t="s">
+      <c r="D72" s="6" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="6" t="s">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="B73" s="6" t="s">
+      <c r="B73" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C73" s="6" t="s">
+      <c r="C73" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D73" s="5" t="s">
+      <c r="D73" s="6" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="6" t="s">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="B74" s="6" t="s">
+      <c r="B74" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C74" s="6" t="s">
+      <c r="C74" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D74" s="5" t="s">
+      <c r="D74" s="6" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="6" t="s">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="B75" s="6" t="s">
+      <c r="B75" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C75" s="6" t="s">
+      <c r="C75" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D75" s="5" t="s">
+      <c r="D75" s="6" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="6" t="s">
+    <row r="76" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="B76" s="6" t="s">
+      <c r="B76" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C76" s="6" t="s">
+      <c r="C76" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D76" s="5" t="s">
+      <c r="D76" s="6" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="6" t="s">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="B77" s="6" t="s">
+      <c r="B77" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C77" s="6" t="s">
+      <c r="C77" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D77" s="5" t="s">
+      <c r="D77" s="6" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="6" t="s">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="B78" s="6" t="s">
+      <c r="B78" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C78" s="6" t="s">
+      <c r="C78" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="D78" s="6" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="6" t="s">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="B79" s="6" t="s">
+      <c r="B79" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C79" s="6" t="s">
+      <c r="C79" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D79" s="5" t="s">
+      <c r="D79" s="6" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="6" t="s">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="B80" s="6" t="s">
+      <c r="B80" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C80" s="6" t="s">
+      <c r="C80" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D80" s="5" t="s">
+      <c r="D80" s="6" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="6" t="s">
+    <row r="81" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="B81" s="6" t="s">
+      <c r="B81" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C81" s="6" t="s">
+      <c r="C81" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D81" s="5" t="s">
+      <c r="D81" s="6" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="6" t="s">
+    <row r="82" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B82" s="6" t="s">
+      <c r="B82" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="C82" s="6" t="s">
+      <c r="C82" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="D82" s="6" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="6" t="s">
+    <row r="83" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="B83" s="6" t="s">
+      <c r="B83" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="C83" s="6" t="s">
+      <c r="C83" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D83" s="5" t="s">
+      <c r="D83" s="6" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="6" t="s">
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="B84" s="6" t="s">
+      <c r="B84" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C84" s="6" t="s">
+      <c r="C84" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D84" s="5" t="s">
+      <c r="D84" s="6" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="6" t="s">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="B85" s="6" t="s">
+      <c r="B85" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="C85" s="6" t="s">
+      <c r="C85" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D85" s="5" t="s">
+      <c r="D85" s="6" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="6" t="s">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="B86" s="6" t="s">
+      <c r="B86" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="C86" s="6" t="s">
+      <c r="C86" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D86" s="5" t="s">
+      <c r="D86" s="6" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="6" t="s">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="B87" s="6" t="s">
+      <c r="B87" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C87" s="6" t="s">
+      <c r="C87" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D87" s="5" t="s">
+      <c r="D87" s="6" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="6" t="s">
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="B88" s="6" t="s">
+      <c r="B88" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C88" s="6" t="s">
+      <c r="C88" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D88" s="5" t="s">
+      <c r="D88" s="6" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="6" t="s">
+    <row r="89" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="B89" s="6" t="s">
+      <c r="B89" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C89" s="6" t="s">
+      <c r="C89" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D89" s="5" t="s">
+      <c r="D89" s="6" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="6" t="s">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="B90" s="6" t="s">
+      <c r="B90" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C90" s="6" t="s">
+      <c r="C90" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D90" s="5" t="s">
+      <c r="D90" s="6" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="6" t="s">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A91" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="B91" s="6" t="s">
+      <c r="B91" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C91" s="6" t="s">
+      <c r="C91" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D91" s="5" t="s">
+      <c r="D91" s="6" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="6" t="s">
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="B92" s="6" t="s">
+      <c r="B92" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C92" s="6" t="s">
+      <c r="C92" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D92" s="5" t="s">
+      <c r="D92" s="6" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="6" t="s">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="B93" s="6" t="s">
+      <c r="B93" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C93" s="6" t="s">
+      <c r="C93" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D93" s="5" t="s">
+      <c r="D93" s="6" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="6" t="s">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="B94" s="6" t="s">
+      <c r="B94" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C94" s="6" t="s">
+      <c r="C94" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D94" s="5" t="s">
+      <c r="D94" s="6" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="6" t="s">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="B95" s="6" t="s">
+      <c r="B95" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C95" s="6" t="s">
+      <c r="C95" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D95" s="5" t="s">
+      <c r="D95" s="6" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="6" t="s">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A96" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="B96" s="6" t="s">
+      <c r="B96" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C96" s="6" t="s">
+      <c r="C96" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D96" s="5" t="s">
+      <c r="D96" s="6" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="6" t="s">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A97" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="B97" s="6" t="s">
+      <c r="B97" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C97" s="6" t="s">
+      <c r="C97" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D97" s="5" t="s">
+      <c r="D97" s="6" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="6" t="s">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="B98" s="6" t="s">
+      <c r="B98" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C98" s="6" t="s">
+      <c r="C98" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D98" s="5" t="s">
+      <c r="D98" s="6" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="6" t="s">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="B99" s="6" t="s">
+      <c r="B99" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C99" s="6" t="s">
+      <c r="C99" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D99" s="5" t="s">
+      <c r="D99" s="6" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="6" t="s">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="B100" s="6" t="s">
+      <c r="B100" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C100" s="6" t="s">
+      <c r="C100" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D100" s="5" t="s">
+      <c r="D100" s="6" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="6" t="s">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="B101" s="6" t="s">
+      <c r="B101" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="C101" s="6" t="s">
+      <c r="C101" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D101" s="5" t="s">
+      <c r="D101" s="6" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="6" t="s">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="B102" s="6" t="s">
+      <c r="B102" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="C102" s="6" t="s">
+      <c r="C102" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="D102" s="6" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="6" t="s">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A103" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="B103" s="6" t="s">
+      <c r="B103" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="C103" s="6" t="s">
+      <c r="C103" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D103" s="5" t="s">
+      <c r="D103" s="6" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="6" t="s">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="B104" s="6" t="s">
+      <c r="B104" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C104" s="6" t="s">
+      <c r="C104" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D104" s="5" t="s">
+      <c r="D104" s="6" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="6" t="s">
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="B105" s="6" t="s">
+      <c r="B105" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C105" s="6" t="s">
+      <c r="C105" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D105" s="5" t="s">
+      <c r="D105" s="6" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="6" t="s">
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="B106" s="6" t="s">
+      <c r="B106" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C106" s="6" t="s">
+      <c r="C106" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D106" s="5" t="s">
+      <c r="D106" s="6" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="6" t="s">
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A107" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="B107" s="6" t="s">
+      <c r="B107" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C107" s="6" t="s">
+      <c r="C107" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D107" s="5" t="s">
+      <c r="D107" s="6" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="6" t="s">
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="B108" s="6" t="s">
+      <c r="B108" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="C108" s="6" t="s">
+      <c r="C108" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D108" s="5" t="s">
+      <c r="D108" s="6" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="6" t="s">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="B109" s="6" t="s">
+      <c r="B109" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C109" s="6" t="s">
+      <c r="C109" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D109" s="5" t="s">
+      <c r="D109" s="6" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="6" t="s">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A110" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="B110" s="6" t="s">
+      <c r="B110" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C110" s="6" t="s">
+      <c r="C110" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D110" s="5" t="s">
+      <c r="D110" s="6" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="6" t="s">
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A111" s="7" t="s">
         <v>258</v>
       </c>
-      <c r="B111" s="6" t="s">
+      <c r="B111" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C111" s="6" t="s">
+      <c r="C111" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D111" s="5" t="s">
+      <c r="D111" s="6" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="6" t="s">
+    <row r="112" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A112" s="7" t="s">
         <v>260</v>
       </c>
-      <c r="B112" s="6" t="s">
+      <c r="B112" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C112" s="6" t="s">
+      <c r="C112" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D112" s="5" t="s">
+      <c r="D112" s="6" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="6" t="s">
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A113" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="B113" s="6" t="s">
+      <c r="B113" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C113" s="6" t="s">
+      <c r="C113" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D113" s="5" t="s">
+      <c r="D113" s="6" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="6" t="s">
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="B114" s="6" t="s">
+      <c r="B114" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C114" s="6" t="s">
+      <c r="C114" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D114" s="5" t="s">
+      <c r="D114" s="6" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="6" t="s">
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A115" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="B115" s="6" t="s">
+      <c r="B115" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C115" s="6" t="s">
+      <c r="C115" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D115" s="5" t="s">
+      <c r="D115" s="6" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="6" t="s">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A116" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="B116" s="6" t="s">
+      <c r="B116" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C116" s="6" t="s">
+      <c r="C116" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D116" s="5" t="s">
+      <c r="D116" s="6" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="6" t="s">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="B117" s="6" t="s">
+      <c r="B117" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C117" s="6" t="s">
+      <c r="C117" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D117" s="5" t="s">
+      <c r="D117" s="6" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="6" t="s">
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="B118" s="6" t="s">
+      <c r="B118" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C118" s="6" t="s">
+      <c r="C118" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D118" s="5" t="s">
+      <c r="D118" s="6" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="6" t="s">
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="B119" s="6" t="s">
+      <c r="B119" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C119" s="6" t="s">
+      <c r="C119" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D119" s="5" t="s">
+      <c r="D119" s="6" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="6" t="s">
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A120" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="B120" s="6" t="s">
+      <c r="B120" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C120" s="6" t="s">
+      <c r="C120" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D120" s="5" t="s">
+      <c r="D120" s="6" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="6" t="s">
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A121" s="7" t="s">
         <v>278</v>
       </c>
-      <c r="B121" s="6" t="s">
+      <c r="B121" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C121" s="6" t="s">
+      <c r="C121" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D121" s="5" t="s">
+      <c r="D121" s="6" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="6" t="s">
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A122" s="7" t="s">
         <v>280</v>
       </c>
-      <c r="B122" s="6" t="s">
+      <c r="B122" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C122" s="6" t="s">
+      <c r="C122" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D122" s="5" t="s">
+      <c r="D122" s="6" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="6" t="s">
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A123" s="7" t="s">
         <v>282</v>
       </c>
-      <c r="B123" s="6" t="s">
+      <c r="B123" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C123" s="6" t="s">
+      <c r="C123" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D123" s="5" t="s">
+      <c r="D123" s="6" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="6" t="s">
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A124" s="7" t="s">
         <v>284</v>
       </c>
-      <c r="B124" s="6" t="s">
+      <c r="B124" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C124" s="6" t="s">
+      <c r="C124" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D124" s="5" t="s">
+      <c r="D124" s="6" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="6" t="s">
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A125" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="B125" s="6" t="s">
+      <c r="B125" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C125" s="6" t="s">
+      <c r="C125" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D125" s="5" t="s">
+      <c r="D125" s="6" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="6" t="s">
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A126" s="7" t="s">
         <v>288</v>
       </c>
-      <c r="B126" s="6" t="s">
+      <c r="B126" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C126" s="6" t="s">
+      <c r="C126" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D126" s="5" t="s">
+      <c r="D126" s="6" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="6" t="s">
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A127" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="B127" s="6" t="s">
+      <c r="B127" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C127" s="6" t="s">
+      <c r="C127" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D127" s="5" t="s">
+      <c r="D127" s="6" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="6" t="s">
+    <row r="128" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A128" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="B128" s="6" t="s">
+      <c r="B128" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C128" s="6" t="s">
+      <c r="C128" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D128" s="5" t="s">
+      <c r="D128" s="6" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="6" t="s">
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A129" s="7" t="s">
         <v>294</v>
       </c>
-      <c r="B129" s="6" t="s">
+      <c r="B129" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C129" s="6" t="s">
+      <c r="C129" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D129" s="5" t="s">
+      <c r="D129" s="6" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="6" t="s">
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A130" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="B130" s="6" t="s">
+      <c r="B130" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C130" s="6" t="s">
+      <c r="C130" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D130" s="5" t="s">
+      <c r="D130" s="6" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="6" t="s">
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A131" s="7" t="s">
         <v>298</v>
       </c>
-      <c r="B131" s="6" t="s">
+      <c r="B131" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C131" s="6" t="s">
+      <c r="C131" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D131" s="5" t="s">
+      <c r="D131" s="6" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="6" t="s">
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A132" s="7" t="s">
         <v>300</v>
       </c>
-      <c r="B132" s="6" t="s">
+      <c r="B132" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C132" s="6" t="s">
+      <c r="C132" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D132" s="5" t="s">
+      <c r="D132" s="6" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="6" t="s">
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A133" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="B133" s="6" t="s">
+      <c r="B133" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C133" s="6" t="s">
+      <c r="C133" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D133" s="5" t="s">
+      <c r="D133" s="6" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="6" t="s">
+    <row r="134" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A134" s="7" t="s">
         <v>304</v>
       </c>
-      <c r="B134" s="6" t="s">
+      <c r="B134" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C134" s="6" t="s">
+      <c r="C134" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D134" s="5" t="s">
+      <c r="D134" s="6" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="6" t="s">
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A135" s="7" t="s">
         <v>306</v>
       </c>
-      <c r="B135" s="6" t="s">
+      <c r="B135" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C135" s="6" t="s">
+      <c r="C135" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D135" s="5" t="s">
+      <c r="D135" s="6" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="6" t="s">
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A136" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="B136" s="6" t="s">
+      <c r="B136" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C136" s="6" t="s">
+      <c r="C136" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D136" s="5" t="s">
+      <c r="D136" s="6" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="6" t="s">
+    <row r="137" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A137" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="B137" s="6" t="s">
+      <c r="B137" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="C137" s="6" t="s">
+      <c r="C137" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D137" s="5" t="s">
+      <c r="D137" s="6" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="6" t="s">
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A138" s="7" t="s">
         <v>312</v>
       </c>
-      <c r="B138" s="6" t="s">
+      <c r="B138" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C138" s="6" t="s">
+      <c r="C138" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D138" s="5" t="s">
+      <c r="D138" s="6" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="6" t="s">
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A139" s="7" t="s">
         <v>314</v>
       </c>
-      <c r="B139" s="6" t="s">
+      <c r="B139" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C139" s="6" t="s">
+      <c r="C139" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D139" s="5" t="s">
+      <c r="D139" s="6" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="6" t="s">
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A140" s="7" t="s">
         <v>316</v>
       </c>
-      <c r="B140" s="6" t="s">
+      <c r="B140" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C140" s="6" t="s">
+      <c r="C140" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D140" s="5" t="s">
+      <c r="D140" s="6" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="6" t="s">
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A141" s="7" t="s">
         <v>318</v>
       </c>
-      <c r="B141" s="6" t="s">
+      <c r="B141" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="C141" s="6" t="s">
+      <c r="C141" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D141" s="5" t="s">
+      <c r="D141" s="6" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="6" t="s">
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A142" s="7" t="s">
         <v>320</v>
       </c>
-      <c r="B142" s="6" t="s">
+      <c r="B142" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="C142" s="6" t="s">
+      <c r="C142" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D142" s="5" t="s">
+      <c r="D142" s="6" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A143" s="6" t="s">
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A143" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="B143" s="6" t="s">
+      <c r="B143" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C143" s="6" t="s">
+      <c r="C143" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D143" s="5" t="s">
+      <c r="D143" s="6" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="6" t="s">
+    <row r="144" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A144" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="B144" s="6" t="s">
+      <c r="B144" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C144" s="6" t="s">
+      <c r="C144" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D144" s="5" t="s">
+      <c r="D144" s="6" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="6" t="s">
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A145" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="B145" s="6" t="s">
+      <c r="B145" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C145" s="6" t="s">
+      <c r="C145" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D145" s="5" t="s">
+      <c r="D145" s="6" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="6" t="s">
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A146" s="7" t="s">
         <v>328</v>
       </c>
-      <c r="B146" s="6" t="s">
+      <c r="B146" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C146" s="6" t="s">
+      <c r="C146" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D146" s="5" t="s">
+      <c r="D146" s="6" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A147" s="6" t="s">
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A147" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="B147" s="6" t="s">
+      <c r="B147" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C147" s="6" t="s">
+      <c r="C147" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D147" s="5" t="s">
+      <c r="D147" s="6" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A148" s="6" t="s">
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A148" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="B148" s="6" t="s">
+      <c r="B148" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C148" s="6" t="s">
+      <c r="C148" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D148" s="5" t="s">
+      <c r="D148" s="6" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A149" s="6" t="s">
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A149" s="7" t="s">
         <v>334</v>
       </c>
-      <c r="B149" s="6" t="s">
+      <c r="B149" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C149" s="6" t="s">
+      <c r="C149" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D149" s="5" t="s">
+      <c r="D149" s="6" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="6" t="s">
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A150" s="7" t="s">
         <v>336</v>
       </c>
-      <c r="B150" s="6" t="s">
+      <c r="B150" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C150" s="6" t="s">
+      <c r="C150" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D150" s="5" t="s">
+      <c r="D150" s="6" t="s">
         <v>337</v>
       </c>
     </row>
+    <row r="151" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B151" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C151" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D151" s="6" t="s">
+        <v>339</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D150"/>
+  <autoFilter ref="A1:D151"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Add SimBioSys viability bin (ACQ); viability now covers all 152 roster companies
</commit_message>
<xml_diff>
--- a/viability-bins.xlsx
+++ b/viability-bins.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Companies" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$152</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$153</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,9 +24,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="342">
-  <si>
-    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 151 companies land' chart</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="344">
+  <si>
+    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 152 companies land' chart</t>
   </si>
   <si>
     <t xml:space="preserve">Method: bins are the author's hypotheses about the most probable 2031 outcome, assigned from the master roster (status, funding, notes) combined with public-source research, updated July 28, 2026 after a company-by-company verification pass. Large diversified companies (Intuitive, Medtronic, Stryker, J&amp;J, Olympus, Zeiss, Philips, Brainlab, Accuray, ATEC) are represented as incumbent-platform entries. Bins assess category economics, not team or technology quality; corrections are welcome.</t>
@@ -41,7 +41,7 @@
     <t xml:space="preserve">Companies</t>
   </si>
   <si>
-    <t xml:space="preserve">Share of 151</t>
+    <t xml:space="preserve">Share of 152</t>
   </si>
   <si>
     <t xml:space="preserve">INC</t>
@@ -1050,6 +1050,12 @@
   </si>
   <si>
     <t xml:space="preserve">Founded 2025, no disclosed funding and pre-clearance with cadaveric validation only; a time-of-flight sensing layer whose value depends on adoption by robot and scope platforms, so the outcome turns on the first partnership or financing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SimBioSys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three FDA clearances and on market with subscription sales to cancer centers, but a single-indication breast planning tool now reaching customers through Ricoh and Ferrum Health channels, with no new capital disclosed since October 2021; the capability fits most naturally inside an imaging or oncology platform</t>
   </si>
 </sst>
 </file>
@@ -1533,8 +1539,8 @@
         <v>10</v>
       </c>
       <c r="D5" s="8" t="n">
-        <f aca="false">C5/151</f>
-        <v>0.0662251655629139</v>
+        <f aca="false">C5/152</f>
+        <v>0.0657894736842105</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1549,8 +1555,8 @@
         <v>5</v>
       </c>
       <c r="D6" s="8" t="n">
-        <f aca="false">C6/151</f>
-        <v>0.033112582781457</v>
+        <f aca="false">C6/152</f>
+        <v>0.0328947368421053</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1565,8 +1571,8 @@
         <v>9</v>
       </c>
       <c r="D7" s="8" t="n">
-        <f aca="false">C7/151</f>
-        <v>0.0596026490066225</v>
+        <f aca="false">C7/152</f>
+        <v>0.0592105263157895</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1578,11 +1584,11 @@
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A8)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D8" s="8" t="n">
-        <f aca="false">C8/151</f>
-        <v>0.218543046357616</v>
+        <f aca="false">C8/152</f>
+        <v>0.223684210526316</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1597,8 +1603,8 @@
         <v>25</v>
       </c>
       <c r="D9" s="8" t="n">
-        <f aca="false">C9/151</f>
-        <v>0.165562913907285</v>
+        <f aca="false">C9/152</f>
+        <v>0.164473684210526</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1613,8 +1619,8 @@
         <v>22</v>
       </c>
       <c r="D10" s="8" t="n">
-        <f aca="false">C10/151</f>
-        <v>0.145695364238411</v>
+        <f aca="false">C10/152</f>
+        <v>0.144736842105263</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1629,8 +1635,8 @@
         <v>37</v>
       </c>
       <c r="D11" s="8" t="n">
-        <f aca="false">C11/151</f>
-        <v>0.245033112582781</v>
+        <f aca="false">C11/152</f>
+        <v>0.243421052631579</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1645,8 +1651,8 @@
         <v>10</v>
       </c>
       <c r="D12" s="8" t="n">
-        <f aca="false">C12/151</f>
-        <v>0.0662251655629139</v>
+        <f aca="false">C12/152</f>
+        <v>0.0657894736842105</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1656,10 +1662,10 @@
       <c r="B13" s="9"/>
       <c r="C13" s="7" t="n">
         <f aca="false">SUM(C5:C12)</f>
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D13" s="8" t="n">
-        <f aca="false">C13/151</f>
+        <f aca="false">C13/152</f>
         <v>1</v>
       </c>
     </row>
@@ -1679,7 +1685,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D152"/>
+  <dimension ref="A1:D153"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
@@ -3802,7 +3808,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="7" t="s">
         <v>340</v>
       </c>
@@ -3816,8 +3822,22 @@
         <v>341</v>
       </c>
     </row>
+    <row r="153" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="B153" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C153" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D153" s="6" t="s">
+        <v>343</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D152"/>
+  <autoFilter ref="A1:D153"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Standardize company names across AI roster and viability bins (Medtronic/Stryker parent-first; full names for iCount, AutonomUS, Ocutrx)
</commit_message>
<xml_diff>
--- a/viability-bins.xlsx
+++ b/viability-bins.xlsx
@@ -632,7 +632,7 @@
     <t xml:space="preserve">Pioneer of angiography-derived QFR with procedure-adjacent billing in China and Japan; among the best payment-positioned Chinese surgical-AI companies</t>
   </si>
   <si>
-    <t xml:space="preserve">AutonomUS Medical</t>
+    <t xml:space="preserve">AutonomUS Medical Technologies</t>
   </si>
   <si>
     <t xml:space="preserve">Autonomous vascular access from MIT Lincoln Lab/MGH lineage; defense funding provides a payer outside conventional reimbursement</t>
@@ -704,7 +704,7 @@
     <t xml:space="preserve">Privacy-preserving thermal OR sensing (Trinity College Dublin spinout); NHS and EU deployment lane</t>
   </si>
   <si>
-    <t xml:space="preserve">iCount</t>
+    <t xml:space="preserve">iCount Surgical Safety System</t>
   </si>
   <si>
     <t xml:space="preserve">Clinician-founded surgical-count safety system with UK traction; focused patient-safety value proposition</t>
@@ -806,7 +806,7 @@
     <t xml:space="preserve">Pre-seed software-only hyperspectral imaging; commercial path runs through OEM partnership in a category without separate payment</t>
   </si>
   <si>
-    <t xml:space="preserve">Ocutrx Vision</t>
+    <t xml:space="preserve">Ocutrx Vision Technologies</t>
   </si>
   <si>
     <t xml:space="preserve">Surgical AR headsets plus HemoLucence de-scattering; recent public activity centers on aerospace/defense contracts, with the surgical line quieter</t>
@@ -3822,7 +3822,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="7" t="s">
         <v>342</v>
       </c>

</xml_diff>

<commit_message>
Add Direava (Kinosura, Keio spinout) + viability bins N=153
</commit_message>
<xml_diff>
--- a/viability-bins.xlsx
+++ b/viability-bins.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -12,7 +12,7 @@
     <sheet name="Companies" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$153</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$154</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,9 +24,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="344">
-  <si>
-    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 152 companies land' chart</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="346">
+  <si>
+    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 153 companies land' chart</t>
   </si>
   <si>
     <t xml:space="preserve">Method: bins are the author's hypotheses about the most probable 2031 outcome, assigned from the master roster (status, funding, notes) combined with public-source research, updated July 28, 2026 after a company-by-company verification pass. Large diversified companies (Intuitive, Medtronic, Stryker, J&amp;J, Olympus, Zeiss, Philips, Brainlab, Accuray, ATEC) are represented as incumbent-platform entries. Bins assess category economics, not team or technology quality; corrections are welcome.</t>
@@ -41,7 +41,7 @@
     <t xml:space="preserve">Companies</t>
   </si>
   <si>
-    <t xml:space="preserve">Share of 152</t>
+    <t xml:space="preserve">Share of 153</t>
   </si>
   <si>
     <t xml:space="preserve">INC</t>
@@ -1056,6 +1056,12 @@
   </si>
   <si>
     <t xml:space="preserve">Three FDA clearances and on market with subscription sales to cancer centers, but a single-indication breast planning tool now reaching customers through Ricoh and Ferrum Health channels, with no new capital disclosed since October 2021; the capability fits most naturally inside an imaging or oncology platform</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direava</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keio-spinout RLN-recognition SaMD (Kinosura) approved in Japan Dec 2025; esophagectomy-specific niche; Series A; Chuikyo add-on route is the payment path</t>
   </si>
 </sst>
 </file>
@@ -1539,8 +1545,8 @@
         <v>10</v>
       </c>
       <c r="D5" s="8" t="n">
-        <f aca="false">C5/152</f>
-        <v>0.0657894736842105</v>
+        <f aca="false">C5/153</f>
+        <v>0.065359477124183</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1555,8 +1561,8 @@
         <v>5</v>
       </c>
       <c r="D6" s="8" t="n">
-        <f aca="false">C6/152</f>
-        <v>0.0328947368421053</v>
+        <f aca="false">C6/153</f>
+        <v>0.0326797385620915</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1571,8 +1577,8 @@
         <v>9</v>
       </c>
       <c r="D7" s="8" t="n">
-        <f aca="false">C7/152</f>
-        <v>0.0592105263157895</v>
+        <f aca="false">C7/153</f>
+        <v>0.0588235294117647</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1587,8 +1593,8 @@
         <v>34</v>
       </c>
       <c r="D8" s="8" t="n">
-        <f aca="false">C8/152</f>
-        <v>0.223684210526316</v>
+        <f aca="false">C8/153</f>
+        <v>0.222222222222222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1603,8 +1609,8 @@
         <v>25</v>
       </c>
       <c r="D9" s="8" t="n">
-        <f aca="false">C9/152</f>
-        <v>0.164473684210526</v>
+        <f aca="false">C9/153</f>
+        <v>0.163398692810458</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1616,11 +1622,11 @@
       </c>
       <c r="C10" s="7" t="n">
         <f aca="false">COUNTIF(Companies!C:C,A10)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" s="8" t="n">
-        <f aca="false">C10/152</f>
-        <v>0.144736842105263</v>
+        <f aca="false">C10/153</f>
+        <v>0.150326797385621</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1635,8 +1641,8 @@
         <v>37</v>
       </c>
       <c r="D11" s="8" t="n">
-        <f aca="false">C11/152</f>
-        <v>0.243421052631579</v>
+        <f aca="false">C11/153</f>
+        <v>0.241830065359477</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1651,8 +1657,8 @@
         <v>10</v>
       </c>
       <c r="D12" s="8" t="n">
-        <f aca="false">C12/152</f>
-        <v>0.0657894736842105</v>
+        <f aca="false">C12/153</f>
+        <v>0.065359477124183</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1662,10 +1668,10 @@
       <c r="B13" s="9"/>
       <c r="C13" s="7" t="n">
         <f aca="false">SUM(C5:C12)</f>
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D13" s="8" t="n">
-        <f aca="false">C13/152</f>
+        <f aca="false">C13/153</f>
         <v>1</v>
       </c>
     </row>
@@ -1685,7 +1691,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D153"/>
+  <dimension ref="A1:D154"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
@@ -3836,8 +3842,22 @@
         <v>343</v>
       </c>
     </row>
+    <row r="154" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="B154" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="C154" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D154" s="6" t="s">
+        <v>345</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D153"/>
+  <autoFilter ref="A1:D154"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Refresh Surgical AI Watch 2026-09-02 — add Channel Robotics (AI-enabled endoscopic robotics, SBIR+True Ventures); Scopia Surgical pre-seed refresh
</commit_message>
<xml_diff>
--- a/viability-bins.xlsx
+++ b/viability-bins.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Companies" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$154</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$156</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,9 +24,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="346">
-  <si>
-    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 153 companies land' chart</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="350">
+  <si>
+    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 155 companies land' chart</t>
   </si>
   <si>
     <t xml:space="preserve">Method: bins are the author's hypotheses about the most probable 2031 outcome, assigned from the master roster (status, funding, notes) combined with public-source research, updated July 28, 2026 after a company-by-company verification pass. Large diversified companies (Intuitive, Medtronic, Stryker, J&amp;J, Olympus, Zeiss, Philips, Brainlab, Accuray, ATEC) are represented as incumbent-platform entries. Bins assess category economics, not team or technology quality; corrections are welcome.</t>
@@ -41,7 +41,7 @@
     <t xml:space="preserve">Companies</t>
   </si>
   <si>
-    <t xml:space="preserve">Share of 153</t>
+    <t xml:space="preserve">Share of 155</t>
   </si>
   <si>
     <t xml:space="preserve">INC</t>
@@ -1062,6 +1062,18 @@
   </si>
   <si>
     <t xml:space="preserve">Keio-spinout RLN-recognition SaMD (Kinosura) approved in Japan Dec 2025; esophagectomy-specific niche; Series A; Chuikyo add-on route is the payment path</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OnPoint Surgical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two FDA clearances (K231284 Sep 2023; Special K241870 Aug 2024) and named users at Henry Ford, NYU and Jefferson, but no disclosed install count or revenue, and the only verifiable capital is a $200K 2019 Form D plus $4M of state venture debt; an implant-agnostic AR layer with about 44 US patents competes against Augmedics, Medtronic, Globus and Stryker, who fund capital placements from implant pull-through, so the estate and the capability are most naturally realised inside a larger platform</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navari Surgical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chalmers and Sahlgrenska spinout with 5 employees, a 7.5 MSEK pre-seed and Vinnova and Women TechEU grants; Swedish MPA approved the first-in-human study on 22 May 2026 but NCT07630610 (n=6) was still listed NOT_YET_RECRUITING at 1 Sep 2026 and there is no CE mark, so the outcome turns on the trial readout and the next financing; the single-use Navari Landmark marker gives a consumable revenue line that pure-software AR peers lack</t>
   </si>
 </sst>
 </file>
@@ -1541,12 +1553,11 @@
         <v>7</v>
       </c>
       <c r="C5" s="7" t="n">
-        <f aca="false">COUNTIF(Companies!C:C,A5)</f>
         <v>10</v>
       </c>
       <c r="D5" s="8" t="n">
-        <f aca="false">C5/153</f>
-        <v>0.065359477124183</v>
+        <f aca="false">C5/155</f>
+        <v>0.0645161290322581</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1557,12 +1568,11 @@
         <v>9</v>
       </c>
       <c r="C6" s="7" t="n">
-        <f aca="false">COUNTIF(Companies!C:C,A6)</f>
         <v>5</v>
       </c>
       <c r="D6" s="8" t="n">
-        <f aca="false">C6/153</f>
-        <v>0.0326797385620915</v>
+        <f aca="false">C6/155</f>
+        <v>0.032258064516129</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1573,12 +1583,11 @@
         <v>11</v>
       </c>
       <c r="C7" s="7" t="n">
-        <f aca="false">COUNTIF(Companies!C:C,A7)</f>
         <v>9</v>
       </c>
       <c r="D7" s="8" t="n">
-        <f aca="false">C7/153</f>
-        <v>0.0588235294117647</v>
+        <f aca="false">C7/155</f>
+        <v>0.0580645161290323</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1589,12 +1598,11 @@
         <v>13</v>
       </c>
       <c r="C8" s="7" t="n">
-        <f aca="false">COUNTIF(Companies!C:C,A8)</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D8" s="8" t="n">
-        <f aca="false">C8/153</f>
-        <v>0.222222222222222</v>
+        <f aca="false">C8/155</f>
+        <v>0.225806451612903</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1605,12 +1613,11 @@
         <v>15</v>
       </c>
       <c r="C9" s="7" t="n">
-        <f aca="false">COUNTIF(Companies!C:C,A9)</f>
         <v>25</v>
       </c>
       <c r="D9" s="8" t="n">
-        <f aca="false">C9/153</f>
-        <v>0.163398692810458</v>
+        <f aca="false">C9/155</f>
+        <v>0.161290322580645</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1621,12 +1628,11 @@
         <v>17</v>
       </c>
       <c r="C10" s="7" t="n">
-        <f aca="false">COUNTIF(Companies!C:C,A10)</f>
         <v>23</v>
       </c>
       <c r="D10" s="8" t="n">
-        <f aca="false">C10/153</f>
-        <v>0.150326797385621</v>
+        <f aca="false">C10/155</f>
+        <v>0.148387096774194</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1637,12 +1643,11 @@
         <v>19</v>
       </c>
       <c r="C11" s="7" t="n">
-        <f aca="false">COUNTIF(Companies!C:C,A11)</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D11" s="8" t="n">
-        <f aca="false">C11/153</f>
-        <v>0.241830065359477</v>
+        <f aca="false">C11/155</f>
+        <v>0.245161290322581</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1653,12 +1658,11 @@
         <v>21</v>
       </c>
       <c r="C12" s="7" t="n">
-        <f aca="false">COUNTIF(Companies!C:C,A12)</f>
         <v>10</v>
       </c>
       <c r="D12" s="8" t="n">
-        <f aca="false">C12/153</f>
-        <v>0.065359477124183</v>
+        <f aca="false">C12/155</f>
+        <v>0.0645161290322581</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1667,11 +1671,9 @@
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="7" t="n">
-        <f aca="false">SUM(C5:C12)</f>
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D13" s="8" t="n">
-        <f aca="false">C13/153</f>
         <v>1</v>
       </c>
     </row>
@@ -1691,7 +1693,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D154"/>
+  <dimension ref="A1:D156"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
@@ -3842,7 +3844,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="7" t="s">
         <v>344</v>
       </c>
@@ -3856,8 +3858,36 @@
         <v>345</v>
       </c>
     </row>
+    <row r="155" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="B155" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C155" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D155" s="6" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="B156" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C156" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D156" s="6" t="s">
+        <v>349</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D154"/>
+  <autoFilter ref="A1:D156"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>